<commit_message>
Rework growth model into explicit business-model paths (partner joins / part-time evenings / homeowner-only)
</commit_message>
<xml_diff>
--- a/business/growth-poam.xlsx
+++ b/business/growth-poam.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth Curve" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POAM" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Business Model Paths" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -230,7 +230,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -380,6 +380,20 @@
     <xf numFmtId="168" fontId="12" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="13" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -633,7 +647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="48" customWidth="1" style="20" min="1" max="1"/>
@@ -754,62 +768,80 @@
     <row r="16">
       <c r="A16" s="29" t="inlineStr">
         <is>
-          <t>Scenario &amp; Profitability Inputs</t>
+          <t>Path &amp; Profitability Inputs</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="30" t="inlineStr">
         <is>
-          <t>Conservative Growth Multiplier (applied to Base plan volumes)</t>
-        </is>
-      </c>
-      <c r="B17" s="31" t="n">
-        <v>0.6</v>
+          <t>Solo Part-Time Hours / Week (evenings, Paths B &amp; C, and Path A before partner joins)</t>
+        </is>
+      </c>
+      <c r="B17" s="63" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="30" t="inlineStr">
         <is>
-          <t>Aggressive Growth Multiplier (applied to Base plan volumes)</t>
-        </is>
-      </c>
-      <c r="B18" s="31" t="n">
-        <v>1.4</v>
+          <t>Two-Person Full-Time Hours / Week (Path A, after partner joins)</t>
+        </is>
+      </c>
+      <c r="B18" s="63" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="30" t="inlineStr">
         <is>
-          <t>Audit / Self-Inspection Gross Margin (%)</t>
-        </is>
-      </c>
-      <c r="B19" s="32" t="n">
-        <v>0.9</v>
+          <t>Partner Join Month (Path A trigger, 1-12)</t>
+        </is>
+      </c>
+      <c r="B19" s="63" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="30" t="inlineStr">
         <is>
-          <t>Hardening Add-On Gross Margin (%)</t>
+          <t>Audit / Self-Inspection Gross Margin (%)</t>
         </is>
       </c>
       <c r="B20" s="32" t="n">
-        <v>0.65</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="30" t="inlineStr">
         <is>
+          <t>Hardening Add-On Gross Margin (%)</t>
+        </is>
+      </c>
+      <c r="B21" s="32" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
           <t>Fixed Monthly Overhead ($)</t>
         </is>
       </c>
-      <c r="B21" s="33" t="n">
+      <c r="B22" s="33" t="n">
         <v>223</v>
       </c>
     </row>
+    <row r="24" ht="55" customHeight="1" s="21">
+      <c r="A24" s="45" t="inlineStr">
+        <is>
+          <t>These three paths are the actual decision on the table, not just optimism levels. Path A assumes your business partner leaves their job once volume justifies it (Month 19 sets when); Path B keeps this a permanent evenings/weekends operation; Path C also stays part-time solo but drops the hardening add-on entirely, which sidesteps almost every open item in legal-risk-notes.md since there's no contractor-licensing exemption being relied on.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A24:F24"/>
     <mergeCell ref="A14:F14"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -1346,7 +1378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -1412,56 +1444,56 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="21">
-      <c r="A4" s="42" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="B4" s="42" t="inlineStr">
+      <c r="A4" s="64" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="B4" s="64" t="inlineStr">
         <is>
           <t>Phase 0 — Pre-Launch</t>
         </is>
       </c>
-      <c r="C4" s="42" t="inlineStr">
-        <is>
-          <t>Form California LLC (Articles of Organization)</t>
-        </is>
-      </c>
-      <c r="D4" s="42" t="inlineStr">
-        <is>
-          <t>Legal</t>
-        </is>
-      </c>
-      <c r="E4" s="42" t="inlineStr">
+      <c r="C4" s="64" t="inlineStr">
+        <is>
+          <t>Decide operating path: (A) partner joins full-time once volume justifies it, (B) permanent part-time evenings solo, or (C) homeowner-inspections-only solo part-time (no hardening add-on)</t>
+        </is>
+      </c>
+      <c r="D4" s="64" t="inlineStr">
+        <is>
+          <t>Planning</t>
+        </is>
+      </c>
+      <c r="E4" s="64" t="inlineStr">
         <is>
           <t>Before Month 1</t>
         </is>
       </c>
-      <c r="F4" s="42" t="inlineStr">
-        <is>
-          <t>Matt</t>
-        </is>
-      </c>
-      <c r="G4" s="42" t="inlineStr">
+      <c r="F4" s="64" t="inlineStr">
+        <is>
+          <t>Matt (+ partner)</t>
+        </is>
+      </c>
+      <c r="G4" s="64" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H4" s="42" t="inlineStr">
+      <c r="H4" s="64" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="I4" s="42" t="inlineStr">
-        <is>
-          <t>LLC registered with CA Secretary of State</t>
+      <c r="I4" s="64" t="inlineStr">
+        <is>
+          <t>Decision documented — see 'Business Model Paths' tab. Determines whether hardening-related POAM items (1.3, 2.1) and legal-risk items 1/2/5/6 are even relevant.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="21">
       <c r="A5" s="42" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="B5" s="42" t="inlineStr">
@@ -1471,12 +1503,12 @@
       </c>
       <c r="C5" s="42" t="inlineStr">
         <is>
-          <t>Obtain EIN + open business bank account</t>
+          <t>Form California LLC (Articles of Organization)</t>
         </is>
       </c>
       <c r="D5" s="42" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="E5" s="42" t="inlineStr">
@@ -1491,7 +1523,7 @@
       </c>
       <c r="G5" s="42" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H5" s="42" t="inlineStr">
@@ -1501,14 +1533,14 @@
       </c>
       <c r="I5" s="42" t="inlineStr">
         <is>
-          <t>EIN issued, account open</t>
+          <t>LLC registered with CA Secretary of State</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="21">
       <c r="A6" s="42" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="B6" s="42" t="inlineStr">
@@ -1518,12 +1550,12 @@
       </c>
       <c r="C6" s="42" t="inlineStr">
         <is>
-          <t>Bind combined GL + E&amp;O insurance policy</t>
+          <t>Obtain EIN + open business bank account</t>
         </is>
       </c>
       <c r="D6" s="42" t="inlineStr">
         <is>
-          <t>Legal/Risk</t>
+          <t>Financial</t>
         </is>
       </c>
       <c r="E6" s="42" t="inlineStr">
@@ -1548,14 +1580,14 @@
       </c>
       <c r="I6" s="42" t="inlineStr">
         <is>
-          <t>Policy active, ~$145/mo confirmed</t>
+          <t>EIN issued, account open</t>
         </is>
       </c>
     </row>
     <row r="7" ht="39.55" customHeight="1" s="21">
       <c r="A7" s="42" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="B7" s="42" t="inlineStr">
@@ -1565,12 +1597,12 @@
       </c>
       <c r="C7" s="42" t="inlineStr">
         <is>
-          <t>Attorney review of Inspection Agreement, Minor Work Contract, Liability Waiver (Section 9 templates)</t>
+          <t>Bind combined GL + E&amp;O insurance policy</t>
         </is>
       </c>
       <c r="D7" s="42" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Legal/Risk</t>
         </is>
       </c>
       <c r="E7" s="42" t="inlineStr">
@@ -1580,12 +1612,12 @@
       </c>
       <c r="F7" s="42" t="inlineStr">
         <is>
-          <t>Matt + CA attorney</t>
+          <t>Matt</t>
         </is>
       </c>
       <c r="G7" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="H7" s="42" t="inlineStr">
@@ -1595,14 +1627,14 @@
       </c>
       <c r="I7" s="42" t="inlineStr">
         <is>
-          <t>Written sign-off before any client signs a contract</t>
+          <t>Policy active, ~$145/mo confirmed</t>
         </is>
       </c>
     </row>
     <row r="8" ht="39.55" customHeight="1" s="21">
       <c r="A8" s="42" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="B8" s="42" t="inlineStr">
@@ -1612,12 +1644,12 @@
       </c>
       <c r="C8" s="42" t="inlineStr">
         <is>
-          <t>Confirm hardening-work permit requirements per target city (Carlsbad, Escondido, Fallbrook, Ramona, Coto de Caza, Silverado Canyon, etc.)</t>
+          <t>Attorney review of Inspection Agreement, Minor Work Contract, Liability Waiver (Section 9 templates)</t>
         </is>
       </c>
       <c r="D8" s="42" t="inlineStr">
         <is>
-          <t>Legal/Compliance</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="E8" s="42" t="inlineStr">
@@ -1627,7 +1659,7 @@
       </c>
       <c r="F8" s="42" t="inlineStr">
         <is>
-          <t>Matt</t>
+          <t>Matt + CA attorney</t>
         </is>
       </c>
       <c r="G8" s="42" t="inlineStr">
@@ -1642,14 +1674,14 @@
       </c>
       <c r="I8" s="42" t="inlineStr">
         <is>
-          <t>B&amp;P §7048 exemption requires NO permit — verify per city before offering hardening add-on</t>
+          <t>Written sign-off before any client signs a contract</t>
         </is>
       </c>
     </row>
     <row r="9" ht="52.2" customHeight="1" s="21">
       <c r="A9" s="42" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="B9" s="42" t="inlineStr">
@@ -1659,12 +1691,12 @@
       </c>
       <c r="C9" s="42" t="inlineStr">
         <is>
-          <t>Confirm marketing/signage won't count as 'holding out as a contractor' under B&amp;P §7048</t>
+          <t>Confirm hardening-work permit requirements per target city (Carlsbad, Escondido, Fallbrook, Ramona, Coto de Caza, Silverado Canyon, etc.)</t>
         </is>
       </c>
       <c r="D9" s="42" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>Legal/Compliance</t>
         </is>
       </c>
       <c r="E9" s="42" t="inlineStr">
@@ -1674,7 +1706,7 @@
       </c>
       <c r="F9" s="42" t="inlineStr">
         <is>
-          <t>Matt + CA attorney</t>
+          <t>Matt</t>
         </is>
       </c>
       <c r="G9" s="42" t="inlineStr">
@@ -1689,14 +1721,14 @@
       </c>
       <c r="I9" s="42" t="inlineStr">
         <is>
-          <t>Flagged risk: worksite banners + hardening-focused branding could void the minor-work exemption — get explicit guidance before Phase 2 signage/marketing</t>
+          <t>B&amp;P §7048 exemption requires NO permit — verify per city before offering hardening add-on</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="21">
       <c r="A10" s="42" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="B10" s="42" t="inlineStr">
@@ -1706,12 +1738,12 @@
       </c>
       <c r="C10" s="42" t="inlineStr">
         <is>
-          <t>Begin NFPA CWMS certification study</t>
+          <t>Confirm marketing/signage won't count as 'holding out as a contractor' under B&amp;P §7048</t>
         </is>
       </c>
       <c r="D10" s="42" t="inlineStr">
         <is>
-          <t>Certification</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="E10" s="42" t="inlineStr">
@@ -1721,7 +1753,7 @@
       </c>
       <c r="F10" s="42" t="inlineStr">
         <is>
-          <t>Matt</t>
+          <t>Matt + CA attorney</t>
         </is>
       </c>
       <c r="G10" s="42" t="inlineStr">
@@ -1736,14 +1768,14 @@
       </c>
       <c r="I10" s="42" t="inlineStr">
         <is>
-          <t>Exam scheduled</t>
+          <t>Flagged risk: worksite banners + hardening-focused branding could void the minor-work exemption — get explicit guidance before Phase 2 signage/marketing</t>
         </is>
       </c>
     </row>
     <row r="11" ht="26.85" customHeight="1" s="21">
       <c r="A11" s="42" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="B11" s="42" t="inlineStr">
@@ -1753,12 +1785,12 @@
       </c>
       <c r="C11" s="42" t="inlineStr">
         <is>
-          <t>Website live with correct pricing ($500/$200) and SoCal geography</t>
+          <t>Begin NFPA CWMS certification study</t>
         </is>
       </c>
       <c r="D11" s="42" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Certification</t>
         </is>
       </c>
       <c r="E11" s="42" t="inlineStr">
@@ -1776,41 +1808,41 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H11" s="43" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="H11" s="42" t="inlineStr">
+        <is>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="I11" s="42" t="inlineStr">
         <is>
-          <t>Completed — charred-guard-site updated</t>
+          <t>Exam scheduled</t>
         </is>
       </c>
     </row>
     <row r="12" ht="26.85" customHeight="1" s="21">
       <c r="A12" s="42" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="B12" s="42" t="inlineStr">
         <is>
-          <t>Phase 1 — Audit-Only Launch (M1-3)</t>
+          <t>Phase 0 — Pre-Launch</t>
         </is>
       </c>
       <c r="C12" s="42" t="inlineStr">
         <is>
-          <t>Deliver first paid on-site audit</t>
+          <t>Website live with correct pricing ($500/$200) and SoCal geography</t>
         </is>
       </c>
       <c r="D12" s="42" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E12" s="42" t="inlineStr">
         <is>
-          <t>Month 1</t>
+          <t>Before Month 1</t>
         </is>
       </c>
       <c r="F12" s="42" t="inlineStr">
@@ -1820,24 +1852,24 @@
       </c>
       <c r="G12" s="42" t="inlineStr">
         <is>
-          <t>0.1-0.4</t>
-        </is>
-      </c>
-      <c r="H12" s="42" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="43" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I12" s="42" t="inlineStr">
         <is>
-          <t>First $500 invoice paid</t>
+          <t>Completed — charred-guard-site updated</t>
         </is>
       </c>
     </row>
     <row r="13" ht="26.85" customHeight="1" s="21">
       <c r="A13" s="42" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="B13" s="42" t="inlineStr">
@@ -1847,7 +1879,7 @@
       </c>
       <c r="C13" s="42" t="inlineStr">
         <is>
-          <t>Deliver first guided self-inspection</t>
+          <t>Deliver first paid on-site audit</t>
         </is>
       </c>
       <c r="D13" s="42" t="inlineStr">
@@ -1877,14 +1909,14 @@
       </c>
       <c r="I13" s="42" t="inlineStr">
         <is>
-          <t>First $200 invoice paid</t>
+          <t>First $500 invoice paid</t>
         </is>
       </c>
     </row>
     <row r="14" ht="26.85" customHeight="1" s="21">
       <c r="A14" s="42" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B14" s="42" t="inlineStr">
@@ -1894,17 +1926,17 @@
       </c>
       <c r="C14" s="42" t="inlineStr">
         <is>
-          <t>Hold hardening add-on revenue until 0.5 and 0.6 are cleared</t>
+          <t>Deliver first guided self-inspection</t>
         </is>
       </c>
       <c r="D14" s="42" t="inlineStr">
         <is>
-          <t>Legal gate</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="E14" s="42" t="inlineStr">
         <is>
-          <t>Months 1-3</t>
+          <t>Month 1</t>
         </is>
       </c>
       <c r="F14" s="42" t="inlineStr">
@@ -1914,7 +1946,7 @@
       </c>
       <c r="G14" s="42" t="inlineStr">
         <is>
-          <t>0.5, 0.6</t>
+          <t>0.1-0.4</t>
         </is>
       </c>
       <c r="H14" s="42" t="inlineStr">
@@ -1924,14 +1956,14 @@
       </c>
       <c r="I14" s="42" t="inlineStr">
         <is>
-          <t>Do not sell hardening work until permit + advertising questions are resolved in writing</t>
+          <t>First $200 invoice paid</t>
         </is>
       </c>
     </row>
     <row r="15" ht="26.85" customHeight="1" s="21">
       <c r="A15" s="42" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B15" s="42" t="inlineStr">
@@ -1941,17 +1973,17 @@
       </c>
       <c r="C15" s="42" t="inlineStr">
         <is>
-          <t>Reach monthly break-even (~$248 revenue covers fixed overhead)</t>
+          <t>Hold hardening add-on revenue until 0.5 and 0.6 are cleared</t>
         </is>
       </c>
       <c r="D15" s="42" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Legal gate</t>
         </is>
       </c>
       <c r="E15" s="42" t="inlineStr">
         <is>
-          <t>Month 3</t>
+          <t>Months 1-3</t>
         </is>
       </c>
       <c r="F15" s="42" t="inlineStr">
@@ -1961,7 +1993,7 @@
       </c>
       <c r="G15" s="42" t="inlineStr">
         <is>
-          <t>1.1, 1.2</t>
+          <t>0.5, 0.6</t>
         </is>
       </c>
       <c r="H15" s="42" t="inlineStr">
@@ -1971,14 +2003,14 @@
       </c>
       <c r="I15" s="42" t="inlineStr">
         <is>
-          <t>See business plan §7.3</t>
+          <t>Do not sell hardening work until permit + advertising questions are resolved in writing</t>
         </is>
       </c>
     </row>
     <row r="16" ht="26.85" customHeight="1" s="21">
       <c r="A16" s="42" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B16" s="42" t="inlineStr">
@@ -1988,17 +2020,17 @@
       </c>
       <c r="C16" s="42" t="inlineStr">
         <is>
-          <t>First conversation with a local independent insurance broker or realtor</t>
+          <t>Reach monthly break-even (~$248 revenue covers fixed overhead)</t>
         </is>
       </c>
       <c r="D16" s="42" t="inlineStr">
         <is>
-          <t>B2B/Marketing</t>
+          <t>Financial</t>
         </is>
       </c>
       <c r="E16" s="42" t="inlineStr">
         <is>
-          <t>Months 1-3</t>
+          <t>Month 3</t>
         </is>
       </c>
       <c r="F16" s="42" t="inlineStr">
@@ -2008,7 +2040,7 @@
       </c>
       <c r="G16" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.1, 1.2</t>
         </is>
       </c>
       <c r="H16" s="42" t="inlineStr">
@@ -2018,34 +2050,34 @@
       </c>
       <c r="I16" s="42" t="inlineStr">
         <is>
-          <t>Relationship opened, not necessarily signed</t>
+          <t>See business plan §7.3</t>
         </is>
       </c>
     </row>
     <row r="17" ht="26.85" customHeight="1" s="21">
       <c r="A17" s="42" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B17" s="42" t="inlineStr">
         <is>
-          <t>Phase 2 — Hardening Launch &amp; Marketing Scale (M4-6)</t>
+          <t>Phase 1 — Audit-Only Launch (M1-3)</t>
         </is>
       </c>
       <c r="C17" s="42" t="inlineStr">
         <is>
-          <t>Turn on hardening add-on revenue</t>
+          <t>First conversation with a local independent insurance broker or realtor</t>
         </is>
       </c>
       <c r="D17" s="42" t="inlineStr">
         <is>
-          <t>Ops/Legal</t>
+          <t>B2B/Marketing</t>
         </is>
       </c>
       <c r="E17" s="42" t="inlineStr">
         <is>
-          <t>Month 4</t>
+          <t>Months 1-3</t>
         </is>
       </c>
       <c r="F17" s="42" t="inlineStr">
@@ -2055,7 +2087,7 @@
       </c>
       <c r="G17" s="42" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H17" s="42" t="inlineStr">
@@ -2065,14 +2097,14 @@
       </c>
       <c r="I17" s="42" t="inlineStr">
         <is>
-          <t>Only after 0.5 and 0.6 are formally cleared</t>
+          <t>Relationship opened, not necessarily signed</t>
         </is>
       </c>
     </row>
     <row r="18" ht="26.85" customHeight="1" s="21">
       <c r="A18" s="42" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="B18" s="42" t="inlineStr">
@@ -2082,12 +2114,12 @@
       </c>
       <c r="C18" s="42" t="inlineStr">
         <is>
-          <t>Launch Nextdoor Verified Sponsorship in 2-3 target ZIP codes</t>
+          <t>Turn on hardening add-on revenue</t>
         </is>
       </c>
       <c r="D18" s="42" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Ops/Legal</t>
         </is>
       </c>
       <c r="E18" s="42" t="inlineStr">
@@ -2102,7 +2134,7 @@
       </c>
       <c r="G18" s="42" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="H18" s="42" t="inlineStr">
@@ -2112,14 +2144,14 @@
       </c>
       <c r="I18" s="42" t="inlineStr">
         <is>
-          <t>Sponsorship live</t>
+          <t>Only after 0.5 and 0.6 are formally cleared</t>
         </is>
       </c>
     </row>
     <row r="19" ht="26.85" customHeight="1" s="21">
       <c r="A19" s="42" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="B19" s="42" t="inlineStr">
@@ -2129,7 +2161,7 @@
       </c>
       <c r="C19" s="42" t="inlineStr">
         <is>
-          <t>Deliver first HOA or Fire Safe Council presentation</t>
+          <t>Launch Nextdoor Verified Sponsorship in 2-3 target ZIP codes</t>
         </is>
       </c>
       <c r="D19" s="42" t="inlineStr">
@@ -2139,7 +2171,7 @@
       </c>
       <c r="E19" s="42" t="inlineStr">
         <is>
-          <t>Months 4-6</t>
+          <t>Month 4</t>
         </is>
       </c>
       <c r="F19" s="42" t="inlineStr">
@@ -2149,7 +2181,7 @@
       </c>
       <c r="G19" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="H19" s="42" t="inlineStr">
@@ -2159,14 +2191,14 @@
       </c>
       <c r="I19" s="42" t="inlineStr">
         <is>
-          <t>Presentation delivered</t>
+          <t>Sponsorship live</t>
         </is>
       </c>
     </row>
     <row r="20" ht="26.85" customHeight="1" s="21">
       <c r="A20" s="42" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="B20" s="42" t="inlineStr">
@@ -2176,12 +2208,12 @@
       </c>
       <c r="C20" s="42" t="inlineStr">
         <is>
-          <t>NFPA CWMS certification achieved</t>
+          <t>Deliver first HOA or Fire Safe Council presentation</t>
         </is>
       </c>
       <c r="D20" s="42" t="inlineStr">
         <is>
-          <t>Certification</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E20" s="42" t="inlineStr">
@@ -2196,7 +2228,7 @@
       </c>
       <c r="G20" s="42" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H20" s="42" t="inlineStr">
@@ -2206,14 +2238,14 @@
       </c>
       <c r="I20" s="42" t="inlineStr">
         <is>
-          <t>Trigger: add certification badge + trust stats to website</t>
+          <t>Presentation delivered</t>
         </is>
       </c>
     </row>
     <row r="21" ht="26.85" customHeight="1" s="21">
       <c r="A21" s="42" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="B21" s="42" t="inlineStr">
@@ -2223,17 +2255,17 @@
       </c>
       <c r="C21" s="42" t="inlineStr">
         <is>
-          <t>First capacity check-in using Growth Curve sheet</t>
+          <t>NFPA CWMS certification achieved</t>
         </is>
       </c>
       <c r="D21" s="42" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>Certification</t>
         </is>
       </c>
       <c r="E21" s="42" t="inlineStr">
         <is>
-          <t>Month 6</t>
+          <t>Months 4-6</t>
         </is>
       </c>
       <c r="F21" s="42" t="inlineStr">
@@ -2243,7 +2275,7 @@
       </c>
       <c r="G21" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="H21" s="42" t="inlineStr">
@@ -2253,34 +2285,34 @@
       </c>
       <c r="I21" s="42" t="inlineStr">
         <is>
-          <t>Confirm Hours/Week is still under the sustainable threshold</t>
+          <t>Trigger: add certification badge + trust stats to website</t>
         </is>
       </c>
     </row>
     <row r="22" ht="26.85" customHeight="1" s="21">
       <c r="A22" s="42" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="B22" s="42" t="inlineStr">
         <is>
-          <t>Phase 3 — Partnerships &amp; Capacity Checkpoint (M7-9)</t>
+          <t>Phase 2 — Hardening Launch &amp; Marketing Scale (M4-6)</t>
         </is>
       </c>
       <c r="C22" s="42" t="inlineStr">
         <is>
-          <t>Signed referral agreement with 1+ insurance broker</t>
+          <t>First capacity check-in using Growth Curve sheet</t>
         </is>
       </c>
       <c r="D22" s="42" t="inlineStr">
         <is>
-          <t>B2B</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="E22" s="42" t="inlineStr">
         <is>
-          <t>Months 7-9</t>
+          <t>Month 6</t>
         </is>
       </c>
       <c r="F22" s="42" t="inlineStr">
@@ -2290,7 +2322,7 @@
       </c>
       <c r="G22" s="42" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H22" s="42" t="inlineStr">
@@ -2300,14 +2332,14 @@
       </c>
       <c r="I22" s="42" t="inlineStr">
         <is>
-          <t>Signed agreement or MOU</t>
+          <t>Confirm Hours/Week is still under the sustainable threshold</t>
         </is>
       </c>
     </row>
     <row r="23" ht="26.85" customHeight="1" s="21">
       <c r="A23" s="42" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B23" s="42" t="inlineStr">
@@ -2317,7 +2349,7 @@
       </c>
       <c r="C23" s="42" t="inlineStr">
         <is>
-          <t>Formal referral relationship with 1+ real estate agent (AB-38 angle)</t>
+          <t>Signed referral agreement with 1+ insurance broker</t>
         </is>
       </c>
       <c r="D23" s="42" t="inlineStr">
@@ -2354,7 +2386,7 @@
     <row r="24" ht="39.55" customHeight="1" s="21">
       <c r="A24" s="42" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B24" s="42" t="inlineStr">
@@ -2364,12 +2396,12 @@
       </c>
       <c r="C24" s="42" t="inlineStr">
         <is>
-          <t>Capacity decision: bring on part-time help if Growth Curve sheet shows Hours/Week over threshold</t>
+          <t>Formal referral relationship with 1+ real estate agent (AB-38 angle)</t>
         </is>
       </c>
       <c r="D24" s="42" t="inlineStr">
         <is>
-          <t>Hiring</t>
+          <t>B2B</t>
         </is>
       </c>
       <c r="E24" s="42" t="inlineStr">
@@ -2384,7 +2416,7 @@
       </c>
       <c r="G24" s="42" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="H24" s="42" t="inlineStr">
@@ -2394,14 +2426,14 @@
       </c>
       <c r="I24" s="42" t="inlineStr">
         <is>
-          <t>Decision documented either way — field assistant for hardening installs, or admin/VA for CRM &amp; scheduling</t>
+          <t>Signed agreement or MOU</t>
         </is>
       </c>
     </row>
     <row r="25" ht="26.85" customHeight="1" s="21">
       <c r="A25" s="42" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="B25" s="42" t="inlineStr">
@@ -2411,12 +2443,12 @@
       </c>
       <c r="C25" s="42" t="inlineStr">
         <is>
-          <t>Add a business phone number to the site</t>
+          <t>Capacity decision: bring on part-time help if Growth Curve sheet shows Hours/Week over threshold</t>
         </is>
       </c>
       <c r="D25" s="42" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Hiring</t>
         </is>
       </c>
       <c r="E25" s="42" t="inlineStr">
@@ -2431,7 +2463,7 @@
       </c>
       <c r="G25" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="H25" s="42" t="inlineStr">
@@ -2441,34 +2473,34 @@
       </c>
       <c r="I25" s="42" t="inlineStr">
         <is>
-          <t>Flagged in earlier competitive review</t>
+          <t>Decision documented either way — field assistant for hardening installs, or admin/VA for CRM &amp; scheduling</t>
         </is>
       </c>
     </row>
     <row r="26" ht="39.55" customHeight="1" s="21">
       <c r="A26" s="42" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="B26" s="42" t="inlineStr">
         <is>
-          <t>Phase 4 — Scale &amp; Year 2 Planning (M10-12)</t>
+          <t>Phase 3 — Partnerships &amp; Capacity Checkpoint (M7-9)</t>
         </is>
       </c>
       <c r="C26" s="42" t="inlineStr">
         <is>
-          <t>Reassess whether hardening volume still fits the $1,000 minor-work exemption, or whether a specialty contractor license makes sense</t>
+          <t>Add a business phone number to the site</t>
         </is>
       </c>
       <c r="D26" s="42" t="inlineStr">
         <is>
-          <t>Legal/Ops</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="E26" s="42" t="inlineStr">
         <is>
-          <t>Months 10-12</t>
+          <t>Months 7-9</t>
         </is>
       </c>
       <c r="F26" s="42" t="inlineStr">
@@ -2478,7 +2510,7 @@
       </c>
       <c r="G26" s="42" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" s="42" t="inlineStr">
@@ -2488,14 +2520,14 @@
       </c>
       <c r="I26" s="42" t="inlineStr">
         <is>
-          <t>Written decision + attorney check-in if volume grew</t>
+          <t>Flagged in earlier competitive review</t>
         </is>
       </c>
     </row>
     <row r="27" ht="26.85" customHeight="1" s="21">
       <c r="A27" s="42" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="B27" s="42" t="inlineStr">
@@ -2505,12 +2537,12 @@
       </c>
       <c r="C27" s="42" t="inlineStr">
         <is>
-          <t>Evaluate hiring a second inspector/technician</t>
+          <t>Reassess whether hardening volume still fits the $1,000 minor-work exemption, or whether a specialty contractor license makes sense</t>
         </is>
       </c>
       <c r="D27" s="42" t="inlineStr">
         <is>
-          <t>Hiring</t>
+          <t>Legal/Ops</t>
         </is>
       </c>
       <c r="E27" s="42" t="inlineStr">
@@ -2535,14 +2567,14 @@
       </c>
       <c r="I27" s="42" t="inlineStr">
         <is>
-          <t>Decision documented</t>
+          <t>Written decision + attorney check-in if volume grew</t>
         </is>
       </c>
     </row>
     <row r="28" ht="26.85" customHeight="1" s="21">
       <c r="A28" s="42" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="B28" s="42" t="inlineStr">
@@ -2552,17 +2584,17 @@
       </c>
       <c r="C28" s="42" t="inlineStr">
         <is>
-          <t>Full-year financials reviewed against Year-1 projections</t>
+          <t>Evaluate hiring a second inspector/technician</t>
         </is>
       </c>
       <c r="D28" s="42" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Hiring</t>
         </is>
       </c>
       <c r="E28" s="42" t="inlineStr">
         <is>
-          <t>Month 12</t>
+          <t>Months 10-12</t>
         </is>
       </c>
       <c r="F28" s="42" t="inlineStr">
@@ -2572,7 +2604,7 @@
       </c>
       <c r="G28" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="H28" s="42" t="inlineStr">
@@ -2582,52 +2614,99 @@
       </c>
       <c r="I28" s="42" t="inlineStr">
         <is>
-          <t>Actuals vs. plan variance noted</t>
+          <t>Decision documented</t>
         </is>
       </c>
     </row>
     <row r="29" ht="26.85" customHeight="1" s="21">
       <c r="A29" s="42" t="inlineStr">
         <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="B29" s="42" t="inlineStr">
+        <is>
+          <t>Phase 4 — Scale &amp; Year 2 Planning (M10-12)</t>
+        </is>
+      </c>
+      <c r="C29" s="42" t="inlineStr">
+        <is>
+          <t>Full-year financials reviewed against Year-1 projections</t>
+        </is>
+      </c>
+      <c r="D29" s="42" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
+      <c r="E29" s="42" t="inlineStr">
+        <is>
+          <t>Month 12</t>
+        </is>
+      </c>
+      <c r="F29" s="42" t="inlineStr">
+        <is>
+          <t>Matt</t>
+        </is>
+      </c>
+      <c r="G29" s="42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H29" s="42" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I29" s="42" t="inlineStr">
+        <is>
+          <t>Actuals vs. plan variance noted</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="42" t="inlineStr">
+        <is>
           <t>4.4</t>
         </is>
       </c>
-      <c r="B29" s="42" t="inlineStr">
+      <c r="B30" s="42" t="inlineStr">
         <is>
           <t>Phase 4 — Scale &amp; Year 2 Planning (M10-12)</t>
         </is>
       </c>
-      <c r="C29" s="42" t="inlineStr">
+      <c r="C30" s="42" t="inlineStr">
         <is>
           <t>Draft Year 2 plan and budget</t>
         </is>
       </c>
-      <c r="D29" s="42" t="inlineStr">
+      <c r="D30" s="42" t="inlineStr">
         <is>
           <t>Planning</t>
         </is>
       </c>
-      <c r="E29" s="42" t="inlineStr">
+      <c r="E30" s="42" t="inlineStr">
         <is>
           <t>Month 12</t>
         </is>
       </c>
-      <c r="F29" s="42" t="inlineStr">
+      <c r="F30" s="42" t="inlineStr">
         <is>
           <t>Matt</t>
         </is>
       </c>
-      <c r="G29" s="42" t="inlineStr">
+      <c r="G30" s="42" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="H29" s="42" t="inlineStr">
+      <c r="H30" s="42" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="I29" s="42" t="inlineStr">
+      <c r="I30" s="42" t="inlineStr">
         <is>
           <t>Year 2 document drafted</t>
         </is>
@@ -2637,10 +2716,13 @@
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="H4:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list" errorStyle="stop" operator="between">
       <formula1>"Not Started,In Progress,Blocked,Done"</formula1>
       <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation sqref="H4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Not Started,In Progress,Blocked,Done"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -2655,7 +2737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V28"/>
+  <dimension ref="A1:S29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="21" min="1" max="1"/>
@@ -2665,52 +2747,49 @@
     <col width="11" customWidth="1" style="21" min="5" max="5"/>
     <col width="11" customWidth="1" style="21" min="6" max="6"/>
     <col width="11" customWidth="1" style="21" min="7" max="7"/>
-    <col width="11" customWidth="1" style="21" min="8" max="8"/>
-    <col width="3" customWidth="1" style="21" min="9" max="9"/>
+    <col width="3" customWidth="1" style="21" min="8" max="8"/>
+    <col width="11" customWidth="1" style="21" min="9" max="9"/>
     <col width="11" customWidth="1" style="21" min="10" max="10"/>
     <col width="11" customWidth="1" style="21" min="11" max="11"/>
     <col width="11" customWidth="1" style="21" min="12" max="12"/>
     <col width="11" customWidth="1" style="21" min="13" max="13"/>
-    <col width="11" customWidth="1" style="21" min="14" max="14"/>
+    <col width="3" customWidth="1" style="21" min="14" max="14"/>
     <col width="11" customWidth="1" style="21" min="15" max="15"/>
-    <col width="3" customWidth="1" style="21" min="16" max="16"/>
+    <col width="11" customWidth="1" style="21" min="16" max="16"/>
     <col width="11" customWidth="1" style="21" min="17" max="17"/>
     <col width="11" customWidth="1" style="21" min="18" max="18"/>
     <col width="11" customWidth="1" style="21" min="19" max="19"/>
-    <col width="11" customWidth="1" style="21" min="20" max="20"/>
-    <col width="11" customWidth="1" style="21" min="21" max="21"/>
-    <col width="11" customWidth="1" style="21" min="22" max="22"/>
-    <col width="3" customWidth="1" style="21" min="23" max="23"/>
+    <col width="3" customWidth="1" style="21" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="44" t="inlineStr">
         <is>
-          <t>Year 1 Scenarios — Conservative / Base / Aggressive, side by side</t>
+          <t>Which Path — Partner Joins Full-Time / Part-Time Evenings / Homeowner-Only</t>
         </is>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1" s="21">
       <c r="A2" s="45" t="inlineStr">
         <is>
-          <t>Base volumes pull from the Growth Curve tab (the original business-plan numbers). Conservative and Aggressive scale those by the multipliers on the Assumptions tab — change a multiplier and every number below recalculates.</t>
+          <t>Audits / Self / Hardening are editable per-path inputs (blue) — each path has a genuinely different volume story, not just a multiplier. Revenue, Hours/Week, and Capacity are formulas that recalc from the Assumptions tab.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="C4" s="46" t="inlineStr">
-        <is>
-          <t>CONSERVATIVE</t>
-        </is>
-      </c>
-      <c r="J4" s="46" t="inlineStr">
-        <is>
-          <t>BASE (business plan)</t>
-        </is>
-      </c>
-      <c r="Q4" s="46" t="inlineStr">
-        <is>
-          <t>AGGRESSIVE</t>
+      <c r="C4" s="65" t="inlineStr">
+        <is>
+          <t>A — PARTNER JOINS FULL-TIME</t>
+        </is>
+      </c>
+      <c r="I4" s="65" t="inlineStr">
+        <is>
+          <t>B — PART-TIME EVENINGS (SOLO, INDEFINITELY)</t>
+        </is>
+      </c>
+      <c r="O4" s="65" t="inlineStr">
+        <is>
+          <t>C — HOMEOWNER INSPECTIONS ONLY (SOLO, PART-TIME, NO HARDENING)</t>
         </is>
       </c>
     </row>
@@ -2725,1097 +2804,806 @@
           <t>Target Month</t>
         </is>
       </c>
-      <c r="C5" s="48" t="inlineStr">
+      <c r="C5" s="66" t="inlineStr">
         <is>
           <t>Audits</t>
         </is>
       </c>
-      <c r="D5" s="48" t="inlineStr">
+      <c r="D5" s="66" t="inlineStr">
         <is>
           <t>Self</t>
         </is>
       </c>
-      <c r="E5" s="48" t="inlineStr">
+      <c r="E5" s="66" t="inlineStr">
         <is>
           <t>Hardening</t>
         </is>
       </c>
-      <c r="F5" s="48" t="inlineStr">
+      <c r="F5" s="66" t="inlineStr">
         <is>
           <t>Revenue ($)</t>
         </is>
       </c>
-      <c r="G5" s="48" t="inlineStr">
+      <c r="G5" s="66" t="inlineStr">
         <is>
           <t>Hrs/Wk</t>
         </is>
       </c>
-      <c r="H5" s="48" t="inlineStr">
-        <is>
-          <t>Capacity</t>
-        </is>
-      </c>
-      <c r="J5" s="49" t="inlineStr">
+      <c r="I5" s="67" t="inlineStr">
         <is>
           <t>Audits</t>
         </is>
       </c>
-      <c r="K5" s="49" t="inlineStr">
+      <c r="J5" s="67" t="inlineStr">
         <is>
           <t>Self</t>
         </is>
       </c>
-      <c r="L5" s="49" t="inlineStr">
+      <c r="K5" s="67" t="inlineStr">
         <is>
           <t>Hardening</t>
         </is>
       </c>
-      <c r="M5" s="49" t="inlineStr">
+      <c r="L5" s="67" t="inlineStr">
         <is>
           <t>Revenue ($)</t>
         </is>
       </c>
-      <c r="N5" s="49" t="inlineStr">
+      <c r="M5" s="67" t="inlineStr">
         <is>
           <t>Hrs/Wk</t>
         </is>
       </c>
-      <c r="O5" s="49" t="inlineStr">
-        <is>
-          <t>Capacity</t>
-        </is>
-      </c>
-      <c r="Q5" s="50" t="inlineStr">
+      <c r="O5" s="68" t="inlineStr">
         <is>
           <t>Audits</t>
         </is>
       </c>
-      <c r="R5" s="50" t="inlineStr">
+      <c r="P5" s="68" t="inlineStr">
         <is>
           <t>Self</t>
         </is>
       </c>
-      <c r="S5" s="50" t="inlineStr">
+      <c r="Q5" s="68" t="inlineStr">
         <is>
           <t>Hardening</t>
         </is>
       </c>
-      <c r="T5" s="50" t="inlineStr">
+      <c r="R5" s="68" t="inlineStr">
         <is>
           <t>Revenue ($)</t>
         </is>
       </c>
-      <c r="U5" s="50" t="inlineStr">
+      <c r="S5" s="68" t="inlineStr">
         <is>
           <t>Hrs/Wk</t>
         </is>
       </c>
-      <c r="V5" s="50" t="inlineStr">
-        <is>
-          <t>Capacity</t>
-        </is>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" s="58" t="n">
+      <c r="A6" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="59">
+      <c r="B6" s="69">
         <f>'Growth Curve'!B5</f>
         <v/>
       </c>
-      <c r="C6" s="58">
-        <f>ROUND('Growth Curve'!C5*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="D6" s="58">
-        <f>ROUND('Growth Curve'!D5*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="E6" s="58">
-        <f>ROUND('Growth Curve'!E5*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="F6" s="60">
+      <c r="C6" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="71">
         <f>C6*Assumptions!$B$5+D6*Assumptions!$B$6+E6*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G6" s="61">
+      <c r="G6" s="72">
         <f>(C6*Assumptions!$B$8+D6*Assumptions!$B$9+E6*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="H6" s="58">
-        <f>IF(G6&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="I6" s="62" t="n"/>
-      <c r="J6" s="58">
-        <f>'Growth Curve'!C5</f>
-        <v/>
-      </c>
-      <c r="K6" s="58">
-        <f>'Growth Curve'!D5</f>
-        <v/>
-      </c>
-      <c r="L6" s="58">
-        <f>'Growth Curve'!E5</f>
-        <v/>
-      </c>
-      <c r="M6" s="60">
-        <f>J6*Assumptions!$B$5+K6*Assumptions!$B$6+L6*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="N6" s="61">
-        <f>(J6*Assumptions!$B$8+K6*Assumptions!$B$9+L6*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="O6" s="58">
-        <f>IF(N6&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="P6" s="62" t="n"/>
-      <c r="Q6" s="58">
-        <f>ROUND('Growth Curve'!C5*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="R6" s="58">
-        <f>ROUND('Growth Curve'!D5*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="S6" s="58">
-        <f>ROUND('Growth Curve'!E5*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="T6" s="60">
-        <f>Q6*Assumptions!$B$5+R6*Assumptions!$B$6+S6*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="U6" s="61">
-        <f>(Q6*Assumptions!$B$8+R6*Assumptions!$B$9+S6*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="V6" s="58">
-        <f>IF(U6&gt;Assumptions!$B$11,"OVER","OK")</f>
+      <c r="I6" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="71">
+        <f>I6*Assumptions!$B$5+J6*Assumptions!$B$6+K6*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="M6" s="72">
+        <f>(I6*Assumptions!$B$8+J6*Assumptions!$B$9+K6*Assumptions!$B$10)/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="O6" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="71">
+        <f>O6*Assumptions!$B$5+P6*Assumptions!$B$6+Q6*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="S6" s="72">
+        <f>(O6*Assumptions!$B$8+P6*Assumptions!$B$9+Q6*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="58" t="n">
+      <c r="A7" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="59">
+      <c r="B7" s="69">
         <f>'Growth Curve'!B6</f>
         <v/>
       </c>
-      <c r="C7" s="58">
-        <f>ROUND('Growth Curve'!C6*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="D7" s="58">
-        <f>ROUND('Growth Curve'!D6*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="E7" s="58">
-        <f>ROUND('Growth Curve'!E6*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="F7" s="60">
+      <c r="C7" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="71">
         <f>C7*Assumptions!$B$5+D7*Assumptions!$B$6+E7*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G7" s="61">
+      <c r="G7" s="72">
         <f>(C7*Assumptions!$B$8+D7*Assumptions!$B$9+E7*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="H7" s="58">
-        <f>IF(G7&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="I7" s="62" t="n"/>
-      <c r="J7" s="58">
-        <f>'Growth Curve'!C6</f>
-        <v/>
-      </c>
-      <c r="K7" s="58">
-        <f>'Growth Curve'!D6</f>
-        <v/>
-      </c>
-      <c r="L7" s="58">
-        <f>'Growth Curve'!E6</f>
-        <v/>
-      </c>
-      <c r="M7" s="60">
-        <f>J7*Assumptions!$B$5+K7*Assumptions!$B$6+L7*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="N7" s="61">
-        <f>(J7*Assumptions!$B$8+K7*Assumptions!$B$9+L7*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="O7" s="58">
-        <f>IF(N7&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="P7" s="62" t="n"/>
-      <c r="Q7" s="58">
-        <f>ROUND('Growth Curve'!C6*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="R7" s="58">
-        <f>ROUND('Growth Curve'!D6*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="S7" s="58">
-        <f>ROUND('Growth Curve'!E6*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="T7" s="60">
-        <f>Q7*Assumptions!$B$5+R7*Assumptions!$B$6+S7*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="U7" s="61">
-        <f>(Q7*Assumptions!$B$8+R7*Assumptions!$B$9+S7*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="V7" s="58">
-        <f>IF(U7&gt;Assumptions!$B$11,"OVER","OK")</f>
+      <c r="I7" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="71">
+        <f>I7*Assumptions!$B$5+J7*Assumptions!$B$6+K7*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="M7" s="72">
+        <f>(I7*Assumptions!$B$8+J7*Assumptions!$B$9+K7*Assumptions!$B$10)/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="O7" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="P7" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="71">
+        <f>O7*Assumptions!$B$5+P7*Assumptions!$B$6+Q7*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="S7" s="72">
+        <f>(O7*Assumptions!$B$8+P7*Assumptions!$B$9+Q7*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="58" t="n">
+      <c r="A8" s="30" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="59">
+      <c r="B8" s="69">
         <f>'Growth Curve'!B7</f>
         <v/>
       </c>
-      <c r="C8" s="58">
-        <f>ROUND('Growth Curve'!C7*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="D8" s="58">
-        <f>ROUND('Growth Curve'!D7*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="E8" s="58">
-        <f>ROUND('Growth Curve'!E7*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="F8" s="60">
+      <c r="C8" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="71">
         <f>C8*Assumptions!$B$5+D8*Assumptions!$B$6+E8*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G8" s="61">
+      <c r="G8" s="72">
         <f>(C8*Assumptions!$B$8+D8*Assumptions!$B$9+E8*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="H8" s="58">
-        <f>IF(G8&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="I8" s="62" t="n"/>
-      <c r="J8" s="58">
-        <f>'Growth Curve'!C7</f>
-        <v/>
-      </c>
-      <c r="K8" s="58">
-        <f>'Growth Curve'!D7</f>
-        <v/>
-      </c>
-      <c r="L8" s="58">
-        <f>'Growth Curve'!E7</f>
-        <v/>
-      </c>
-      <c r="M8" s="60">
-        <f>J8*Assumptions!$B$5+K8*Assumptions!$B$6+L8*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="N8" s="61">
-        <f>(J8*Assumptions!$B$8+K8*Assumptions!$B$9+L8*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="O8" s="58">
-        <f>IF(N8&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="P8" s="62" t="n"/>
-      <c r="Q8" s="58">
-        <f>ROUND('Growth Curve'!C7*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="R8" s="58">
-        <f>ROUND('Growth Curve'!D7*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="S8" s="58">
-        <f>ROUND('Growth Curve'!E7*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="T8" s="60">
-        <f>Q8*Assumptions!$B$5+R8*Assumptions!$B$6+S8*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="U8" s="61">
-        <f>(Q8*Assumptions!$B$8+R8*Assumptions!$B$9+S8*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="V8" s="58">
-        <f>IF(U8&gt;Assumptions!$B$11,"OVER","OK")</f>
+      <c r="I8" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" s="71">
+        <f>I8*Assumptions!$B$5+J8*Assumptions!$B$6+K8*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="M8" s="72">
+        <f>(I8*Assumptions!$B$8+J8*Assumptions!$B$9+K8*Assumptions!$B$10)/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="O8" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="P8" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q8" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="71">
+        <f>O8*Assumptions!$B$5+P8*Assumptions!$B$6+Q8*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="S8" s="72">
+        <f>(O8*Assumptions!$B$8+P8*Assumptions!$B$9+Q8*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="58" t="n">
+      <c r="A9" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="59">
+      <c r="B9" s="69">
         <f>'Growth Curve'!B8</f>
         <v/>
       </c>
-      <c r="C9" s="58">
-        <f>ROUND('Growth Curve'!C8*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="D9" s="58">
-        <f>ROUND('Growth Curve'!D8*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="E9" s="58">
-        <f>ROUND('Growth Curve'!E8*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="F9" s="60">
+      <c r="C9" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="71">
         <f>C9*Assumptions!$B$5+D9*Assumptions!$B$6+E9*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G9" s="61">
+      <c r="G9" s="72">
         <f>(C9*Assumptions!$B$8+D9*Assumptions!$B$9+E9*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="H9" s="58">
-        <f>IF(G9&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="I9" s="62" t="n"/>
-      <c r="J9" s="58">
-        <f>'Growth Curve'!C8</f>
-        <v/>
-      </c>
-      <c r="K9" s="58">
-        <f>'Growth Curve'!D8</f>
-        <v/>
-      </c>
-      <c r="L9" s="58">
-        <f>'Growth Curve'!E8</f>
-        <v/>
-      </c>
-      <c r="M9" s="60">
-        <f>J9*Assumptions!$B$5+K9*Assumptions!$B$6+L9*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="N9" s="61">
-        <f>(J9*Assumptions!$B$8+K9*Assumptions!$B$9+L9*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="O9" s="58">
-        <f>IF(N9&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="P9" s="62" t="n"/>
-      <c r="Q9" s="58">
-        <f>ROUND('Growth Curve'!C8*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="R9" s="58">
-        <f>ROUND('Growth Curve'!D8*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="S9" s="58">
-        <f>ROUND('Growth Curve'!E8*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="T9" s="60">
-        <f>Q9*Assumptions!$B$5+R9*Assumptions!$B$6+S9*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="U9" s="61">
-        <f>(Q9*Assumptions!$B$8+R9*Assumptions!$B$9+S9*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="V9" s="58">
-        <f>IF(U9&gt;Assumptions!$B$11,"OVER","OK")</f>
+      <c r="I9" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" s="71">
+        <f>I9*Assumptions!$B$5+J9*Assumptions!$B$6+K9*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="M9" s="72">
+        <f>(I9*Assumptions!$B$8+J9*Assumptions!$B$9+K9*Assumptions!$B$10)/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="O9" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="P9" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q9" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="71">
+        <f>O9*Assumptions!$B$5+P9*Assumptions!$B$6+Q9*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="S9" s="72">
+        <f>(O9*Assumptions!$B$8+P9*Assumptions!$B$9+Q9*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="58" t="n">
+      <c r="A10" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="59">
+      <c r="B10" s="69">
         <f>'Growth Curve'!B9</f>
         <v/>
       </c>
-      <c r="C10" s="58">
-        <f>ROUND('Growth Curve'!C9*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="D10" s="58">
-        <f>ROUND('Growth Curve'!D9*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="E10" s="58">
-        <f>ROUND('Growth Curve'!E9*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="F10" s="60">
+      <c r="C10" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="71">
         <f>C10*Assumptions!$B$5+D10*Assumptions!$B$6+E10*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G10" s="61">
+      <c r="G10" s="72">
         <f>(C10*Assumptions!$B$8+D10*Assumptions!$B$9+E10*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="H10" s="58">
-        <f>IF(G10&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="I10" s="62" t="n"/>
-      <c r="J10" s="58">
-        <f>'Growth Curve'!C9</f>
-        <v/>
-      </c>
-      <c r="K10" s="58">
-        <f>'Growth Curve'!D9</f>
-        <v/>
-      </c>
-      <c r="L10" s="58">
-        <f>'Growth Curve'!E9</f>
-        <v/>
-      </c>
-      <c r="M10" s="60">
-        <f>J10*Assumptions!$B$5+K10*Assumptions!$B$6+L10*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="N10" s="61">
-        <f>(J10*Assumptions!$B$8+K10*Assumptions!$B$9+L10*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="O10" s="58">
-        <f>IF(N10&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="P10" s="62" t="n"/>
-      <c r="Q10" s="58">
-        <f>ROUND('Growth Curve'!C9*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="R10" s="58">
-        <f>ROUND('Growth Curve'!D9*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="S10" s="58">
-        <f>ROUND('Growth Curve'!E9*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="T10" s="60">
-        <f>Q10*Assumptions!$B$5+R10*Assumptions!$B$6+S10*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="U10" s="61">
-        <f>(Q10*Assumptions!$B$8+R10*Assumptions!$B$9+S10*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="V10" s="58">
-        <f>IF(U10&gt;Assumptions!$B$11,"OVER","OK")</f>
+      <c r="I10" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" s="71">
+        <f>I10*Assumptions!$B$5+J10*Assumptions!$B$6+K10*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="M10" s="72">
+        <f>(I10*Assumptions!$B$8+J10*Assumptions!$B$9+K10*Assumptions!$B$10)/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="O10" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="P10" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q10" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="71">
+        <f>O10*Assumptions!$B$5+P10*Assumptions!$B$6+Q10*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="S10" s="72">
+        <f>(O10*Assumptions!$B$8+P10*Assumptions!$B$9+Q10*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="58" t="n">
+      <c r="A11" s="30" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="59">
+      <c r="B11" s="69">
         <f>'Growth Curve'!B10</f>
         <v/>
       </c>
-      <c r="C11" s="58">
-        <f>ROUND('Growth Curve'!C10*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="D11" s="58">
-        <f>ROUND('Growth Curve'!D10*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="E11" s="58">
-        <f>ROUND('Growth Curve'!E10*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="F11" s="60">
+      <c r="C11" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="D11" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="71">
         <f>C11*Assumptions!$B$5+D11*Assumptions!$B$6+E11*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G11" s="61">
+      <c r="G11" s="72">
         <f>(C11*Assumptions!$B$8+D11*Assumptions!$B$9+E11*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="H11" s="58">
-        <f>IF(G11&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="I11" s="62" t="n"/>
-      <c r="J11" s="58">
-        <f>'Growth Curve'!C10</f>
-        <v/>
-      </c>
-      <c r="K11" s="58">
-        <f>'Growth Curve'!D10</f>
-        <v/>
-      </c>
-      <c r="L11" s="58">
-        <f>'Growth Curve'!E10</f>
-        <v/>
-      </c>
-      <c r="M11" s="60">
-        <f>J11*Assumptions!$B$5+K11*Assumptions!$B$6+L11*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="N11" s="61">
-        <f>(J11*Assumptions!$B$8+K11*Assumptions!$B$9+L11*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="O11" s="58">
-        <f>IF(N11&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="P11" s="62" t="n"/>
-      <c r="Q11" s="58">
-        <f>ROUND('Growth Curve'!C10*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="R11" s="58">
-        <f>ROUND('Growth Curve'!D10*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="S11" s="58">
-        <f>ROUND('Growth Curve'!E10*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="T11" s="60">
-        <f>Q11*Assumptions!$B$5+R11*Assumptions!$B$6+S11*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="U11" s="61">
-        <f>(Q11*Assumptions!$B$8+R11*Assumptions!$B$9+S11*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="V11" s="58">
-        <f>IF(U11&gt;Assumptions!$B$11,"OVER","OK")</f>
+      <c r="I11" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="J11" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="K11" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" s="71">
+        <f>I11*Assumptions!$B$5+J11*Assumptions!$B$6+K11*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="M11" s="72">
+        <f>(I11*Assumptions!$B$8+J11*Assumptions!$B$9+K11*Assumptions!$B$10)/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="O11" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="P11" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q11" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="71">
+        <f>O11*Assumptions!$B$5+P11*Assumptions!$B$6+Q11*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="S11" s="72">
+        <f>(O11*Assumptions!$B$8+P11*Assumptions!$B$9+Q11*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="58" t="n">
+      <c r="A12" s="30" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="59">
+      <c r="B12" s="69">
         <f>'Growth Curve'!B11</f>
         <v/>
       </c>
-      <c r="C12" s="58">
-        <f>ROUND('Growth Curve'!C11*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="D12" s="58">
-        <f>ROUND('Growth Curve'!D11*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="E12" s="58">
-        <f>ROUND('Growth Curve'!E11*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="F12" s="60">
+      <c r="C12" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="D12" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" s="71">
         <f>C12*Assumptions!$B$5+D12*Assumptions!$B$6+E12*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G12" s="61">
+      <c r="G12" s="72">
         <f>(C12*Assumptions!$B$8+D12*Assumptions!$B$9+E12*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="H12" s="58">
-        <f>IF(G12&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="I12" s="62" t="n"/>
-      <c r="J12" s="58">
-        <f>'Growth Curve'!C11</f>
-        <v/>
-      </c>
-      <c r="K12" s="58">
-        <f>'Growth Curve'!D11</f>
-        <v/>
-      </c>
-      <c r="L12" s="58">
-        <f>'Growth Curve'!E11</f>
-        <v/>
-      </c>
-      <c r="M12" s="60">
-        <f>J12*Assumptions!$B$5+K12*Assumptions!$B$6+L12*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="N12" s="61">
-        <f>(J12*Assumptions!$B$8+K12*Assumptions!$B$9+L12*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="O12" s="58">
-        <f>IF(N12&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="P12" s="62" t="n"/>
-      <c r="Q12" s="58">
-        <f>ROUND('Growth Curve'!C11*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="R12" s="58">
-        <f>ROUND('Growth Curve'!D11*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="S12" s="58">
-        <f>ROUND('Growth Curve'!E11*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="T12" s="60">
-        <f>Q12*Assumptions!$B$5+R12*Assumptions!$B$6+S12*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="U12" s="61">
-        <f>(Q12*Assumptions!$B$8+R12*Assumptions!$B$9+S12*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="V12" s="58">
-        <f>IF(U12&gt;Assumptions!$B$11,"OVER","OK")</f>
+      <c r="I12" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="J12" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" s="71">
+        <f>I12*Assumptions!$B$5+J12*Assumptions!$B$6+K12*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="M12" s="72">
+        <f>(I12*Assumptions!$B$8+J12*Assumptions!$B$9+K12*Assumptions!$B$10)/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="O12" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="P12" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q12" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="71">
+        <f>O12*Assumptions!$B$5+P12*Assumptions!$B$6+Q12*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="S12" s="72">
+        <f>(O12*Assumptions!$B$8+P12*Assumptions!$B$9+Q12*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="58" t="n">
+      <c r="A13" s="30" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="59">
+      <c r="B13" s="69">
         <f>'Growth Curve'!B12</f>
         <v/>
       </c>
-      <c r="C13" s="58">
-        <f>ROUND('Growth Curve'!C12*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="D13" s="58">
-        <f>ROUND('Growth Curve'!D12*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="E13" s="58">
-        <f>ROUND('Growth Curve'!E12*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="F13" s="60">
+      <c r="C13" s="70" t="n">
+        <v>9</v>
+      </c>
+      <c r="D13" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="71">
         <f>C13*Assumptions!$B$5+D13*Assumptions!$B$6+E13*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G13" s="61">
+      <c r="G13" s="72">
         <f>(C13*Assumptions!$B$8+D13*Assumptions!$B$9+E13*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="H13" s="58">
-        <f>IF(G13&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="I13" s="62" t="n"/>
-      <c r="J13" s="58">
-        <f>'Growth Curve'!C12</f>
-        <v/>
-      </c>
-      <c r="K13" s="58">
-        <f>'Growth Curve'!D12</f>
-        <v/>
-      </c>
-      <c r="L13" s="58">
-        <f>'Growth Curve'!E12</f>
-        <v/>
-      </c>
-      <c r="M13" s="60">
-        <f>J13*Assumptions!$B$5+K13*Assumptions!$B$6+L13*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="N13" s="61">
-        <f>(J13*Assumptions!$B$8+K13*Assumptions!$B$9+L13*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="O13" s="58">
-        <f>IF(N13&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="P13" s="62" t="n"/>
-      <c r="Q13" s="58">
-        <f>ROUND('Growth Curve'!C12*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="R13" s="58">
-        <f>ROUND('Growth Curve'!D12*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="S13" s="58">
-        <f>ROUND('Growth Curve'!E12*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="T13" s="60">
-        <f>Q13*Assumptions!$B$5+R13*Assumptions!$B$6+S13*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="U13" s="61">
-        <f>(Q13*Assumptions!$B$8+R13*Assumptions!$B$9+S13*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="V13" s="58">
-        <f>IF(U13&gt;Assumptions!$B$11,"OVER","OK")</f>
+      <c r="I13" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="J13" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" s="71">
+        <f>I13*Assumptions!$B$5+J13*Assumptions!$B$6+K13*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="M13" s="72">
+        <f>(I13*Assumptions!$B$8+J13*Assumptions!$B$9+K13*Assumptions!$B$10)/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="O13" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="P13" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q13" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="71">
+        <f>O13*Assumptions!$B$5+P13*Assumptions!$B$6+Q13*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="S13" s="72">
+        <f>(O13*Assumptions!$B$8+P13*Assumptions!$B$9+Q13*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="58" t="n">
+      <c r="A14" s="30" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="59">
+      <c r="B14" s="69">
         <f>'Growth Curve'!B13</f>
         <v/>
       </c>
-      <c r="C14" s="58">
-        <f>ROUND('Growth Curve'!C13*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="D14" s="58">
-        <f>ROUND('Growth Curve'!D13*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="E14" s="58">
-        <f>ROUND('Growth Curve'!E13*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="F14" s="60">
+      <c r="C14" s="70" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" s="71">
         <f>C14*Assumptions!$B$5+D14*Assumptions!$B$6+E14*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G14" s="61">
+      <c r="G14" s="72">
         <f>(C14*Assumptions!$B$8+D14*Assumptions!$B$9+E14*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="H14" s="58">
-        <f>IF(G14&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="I14" s="62" t="n"/>
-      <c r="J14" s="58">
-        <f>'Growth Curve'!C13</f>
-        <v/>
-      </c>
-      <c r="K14" s="58">
-        <f>'Growth Curve'!D13</f>
-        <v/>
-      </c>
-      <c r="L14" s="58">
-        <f>'Growth Curve'!E13</f>
-        <v/>
-      </c>
-      <c r="M14" s="60">
-        <f>J14*Assumptions!$B$5+K14*Assumptions!$B$6+L14*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="N14" s="61">
-        <f>(J14*Assumptions!$B$8+K14*Assumptions!$B$9+L14*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="O14" s="58">
-        <f>IF(N14&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="P14" s="62" t="n"/>
-      <c r="Q14" s="58">
-        <f>ROUND('Growth Curve'!C13*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="R14" s="58">
-        <f>ROUND('Growth Curve'!D13*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="S14" s="58">
-        <f>ROUND('Growth Curve'!E13*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="T14" s="60">
-        <f>Q14*Assumptions!$B$5+R14*Assumptions!$B$6+S14*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="U14" s="61">
-        <f>(Q14*Assumptions!$B$8+R14*Assumptions!$B$9+S14*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="V14" s="58">
-        <f>IF(U14&gt;Assumptions!$B$11,"OVER","OK")</f>
+      <c r="I14" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="J14" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" s="71">
+        <f>I14*Assumptions!$B$5+J14*Assumptions!$B$6+K14*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="M14" s="72">
+        <f>(I14*Assumptions!$B$8+J14*Assumptions!$B$9+K14*Assumptions!$B$10)/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="O14" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="P14" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q14" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="71">
+        <f>O14*Assumptions!$B$5+P14*Assumptions!$B$6+Q14*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="S14" s="72">
+        <f>(O14*Assumptions!$B$8+P14*Assumptions!$B$9+Q14*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="58" t="n">
+      <c r="A15" s="30" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="59">
+      <c r="B15" s="69">
         <f>'Growth Curve'!B14</f>
         <v/>
       </c>
-      <c r="C15" s="58">
-        <f>ROUND('Growth Curve'!C14*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="D15" s="58">
-        <f>ROUND('Growth Curve'!D14*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="E15" s="58">
-        <f>ROUND('Growth Curve'!E14*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="F15" s="60">
+      <c r="C15" s="70" t="n">
+        <v>11</v>
+      </c>
+      <c r="D15" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" s="71">
         <f>C15*Assumptions!$B$5+D15*Assumptions!$B$6+E15*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G15" s="61">
+      <c r="G15" s="72">
         <f>(C15*Assumptions!$B$8+D15*Assumptions!$B$9+E15*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="H15" s="58">
-        <f>IF(G15&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="I15" s="62" t="n"/>
-      <c r="J15" s="58">
-        <f>'Growth Curve'!C14</f>
-        <v/>
-      </c>
-      <c r="K15" s="58">
-        <f>'Growth Curve'!D14</f>
-        <v/>
-      </c>
-      <c r="L15" s="58">
-        <f>'Growth Curve'!E14</f>
-        <v/>
-      </c>
-      <c r="M15" s="60">
-        <f>J15*Assumptions!$B$5+K15*Assumptions!$B$6+L15*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="N15" s="61">
-        <f>(J15*Assumptions!$B$8+K15*Assumptions!$B$9+L15*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="O15" s="58">
-        <f>IF(N15&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="P15" s="62" t="n"/>
-      <c r="Q15" s="58">
-        <f>ROUND('Growth Curve'!C14*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="R15" s="58">
-        <f>ROUND('Growth Curve'!D14*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="S15" s="58">
-        <f>ROUND('Growth Curve'!E14*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="T15" s="60">
-        <f>Q15*Assumptions!$B$5+R15*Assumptions!$B$6+S15*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="U15" s="61">
-        <f>(Q15*Assumptions!$B$8+R15*Assumptions!$B$9+S15*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="V15" s="58">
-        <f>IF(U15&gt;Assumptions!$B$11,"OVER","OK")</f>
+      <c r="I15" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="J15" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" s="71">
+        <f>I15*Assumptions!$B$5+J15*Assumptions!$B$6+K15*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="M15" s="72">
+        <f>(I15*Assumptions!$B$8+J15*Assumptions!$B$9+K15*Assumptions!$B$10)/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="O15" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="P15" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q15" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="71">
+        <f>O15*Assumptions!$B$5+P15*Assumptions!$B$6+Q15*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="S15" s="72">
+        <f>(O15*Assumptions!$B$8+P15*Assumptions!$B$9+Q15*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="58" t="n">
+      <c r="A16" s="30" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="59">
+      <c r="B16" s="69">
         <f>'Growth Curve'!B15</f>
         <v/>
       </c>
-      <c r="C16" s="58">
-        <f>ROUND('Growth Curve'!C15*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="D16" s="58">
-        <f>ROUND('Growth Curve'!D15*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="E16" s="58">
-        <f>ROUND('Growth Curve'!E15*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="F16" s="60">
+      <c r="C16" s="70" t="n">
+        <v>12</v>
+      </c>
+      <c r="D16" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" s="71">
         <f>C16*Assumptions!$B$5+D16*Assumptions!$B$6+E16*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G16" s="61">
+      <c r="G16" s="72">
         <f>(C16*Assumptions!$B$8+D16*Assumptions!$B$9+E16*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="H16" s="58">
-        <f>IF(G16&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="I16" s="62" t="n"/>
-      <c r="J16" s="58">
-        <f>'Growth Curve'!C15</f>
-        <v/>
-      </c>
-      <c r="K16" s="58">
-        <f>'Growth Curve'!D15</f>
-        <v/>
-      </c>
-      <c r="L16" s="58">
-        <f>'Growth Curve'!E15</f>
-        <v/>
-      </c>
-      <c r="M16" s="60">
-        <f>J16*Assumptions!$B$5+K16*Assumptions!$B$6+L16*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="N16" s="61">
-        <f>(J16*Assumptions!$B$8+K16*Assumptions!$B$9+L16*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="O16" s="58">
-        <f>IF(N16&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="P16" s="62" t="n"/>
-      <c r="Q16" s="58">
-        <f>ROUND('Growth Curve'!C15*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="R16" s="58">
-        <f>ROUND('Growth Curve'!D15*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="S16" s="58">
-        <f>ROUND('Growth Curve'!E15*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="T16" s="60">
-        <f>Q16*Assumptions!$B$5+R16*Assumptions!$B$6+S16*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="U16" s="61">
-        <f>(Q16*Assumptions!$B$8+R16*Assumptions!$B$9+S16*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="V16" s="58">
-        <f>IF(U16&gt;Assumptions!$B$11,"OVER","OK")</f>
+      <c r="I16" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="J16" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" s="71">
+        <f>I16*Assumptions!$B$5+J16*Assumptions!$B$6+K16*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="M16" s="72">
+        <f>(I16*Assumptions!$B$8+J16*Assumptions!$B$9+K16*Assumptions!$B$10)/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="O16" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="P16" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q16" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="71">
+        <f>O16*Assumptions!$B$5+P16*Assumptions!$B$6+Q16*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="S16" s="72">
+        <f>(O16*Assumptions!$B$8+P16*Assumptions!$B$9+Q16*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="58" t="n">
+      <c r="A17" s="30" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="59">
+      <c r="B17" s="69">
         <f>'Growth Curve'!B16</f>
         <v/>
       </c>
-      <c r="C17" s="58">
-        <f>ROUND('Growth Curve'!C16*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="D17" s="58">
-        <f>ROUND('Growth Curve'!D16*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="E17" s="58">
-        <f>ROUND('Growth Curve'!E16*Assumptions!$B$17,0)</f>
-        <v/>
-      </c>
-      <c r="F17" s="60">
+      <c r="C17" s="70" t="n">
+        <v>13</v>
+      </c>
+      <c r="D17" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="F17" s="71">
         <f>C17*Assumptions!$B$5+D17*Assumptions!$B$6+E17*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="G17" s="61">
+      <c r="G17" s="72">
         <f>(C17*Assumptions!$B$8+D17*Assumptions!$B$9+E17*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
-      <c r="H17" s="58">
-        <f>IF(G17&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="I17" s="62" t="n"/>
-      <c r="J17" s="58">
-        <f>'Growth Curve'!C16</f>
-        <v/>
-      </c>
-      <c r="K17" s="58">
-        <f>'Growth Curve'!D16</f>
-        <v/>
-      </c>
-      <c r="L17" s="58">
-        <f>'Growth Curve'!E16</f>
-        <v/>
-      </c>
-      <c r="M17" s="60">
-        <f>J17*Assumptions!$B$5+K17*Assumptions!$B$6+L17*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="N17" s="61">
-        <f>(J17*Assumptions!$B$8+K17*Assumptions!$B$9+L17*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="O17" s="58">
-        <f>IF(N17&gt;Assumptions!$B$11,"OVER","OK")</f>
-        <v/>
-      </c>
-      <c r="P17" s="62" t="n"/>
-      <c r="Q17" s="58">
-        <f>ROUND('Growth Curve'!C16*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="R17" s="58">
-        <f>ROUND('Growth Curve'!D16*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="S17" s="58">
-        <f>ROUND('Growth Curve'!E16*Assumptions!$B$18,0)</f>
-        <v/>
-      </c>
-      <c r="T17" s="60">
-        <f>Q17*Assumptions!$B$5+R17*Assumptions!$B$6+S17*Assumptions!$B$7</f>
-        <v/>
-      </c>
-      <c r="U17" s="61">
-        <f>(Q17*Assumptions!$B$8+R17*Assumptions!$B$9+S17*Assumptions!$B$10)/Assumptions!$B$12</f>
-        <v/>
-      </c>
-      <c r="V17" s="58">
-        <f>IF(U17&gt;Assumptions!$B$11,"OVER","OK")</f>
+      <c r="I17" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="J17" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="K17" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" s="71">
+        <f>I17*Assumptions!$B$5+J17*Assumptions!$B$6+K17*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="M17" s="72">
+        <f>(I17*Assumptions!$B$8+J17*Assumptions!$B$9+K17*Assumptions!$B$10)/Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="O17" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="P17" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q17" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="71">
+        <f>O17*Assumptions!$B$5+P17*Assumptions!$B$6+Q17*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="S17" s="72">
+        <f>(O17*Assumptions!$B$8+P17*Assumptions!$B$9+Q17*Assumptions!$B$10)/Assumptions!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="29" t="inlineStr">
         <is>
-          <t>Year-1 Summary Comparison</t>
+          <t>Year-1 Summary</t>
         </is>
       </c>
     </row>
@@ -3827,17 +3615,17 @@
       </c>
       <c r="B20" s="47" t="inlineStr">
         <is>
-          <t>Conservative</t>
+          <t>A — Partner Joins</t>
         </is>
       </c>
       <c r="C20" s="47" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>B — Evenings Only</t>
         </is>
       </c>
       <c r="D20" s="47" t="inlineStr">
         <is>
-          <t>Aggressive</t>
+          <t>C — Homeowner-Only</t>
         </is>
       </c>
     </row>
@@ -3852,11 +3640,11 @@
         <v/>
       </c>
       <c r="C21" s="55">
-        <f>SUM(J6:J17)</f>
+        <f>SUM(I6:I17)</f>
         <v/>
       </c>
       <c r="D21" s="55">
-        <f>SUM(Q6:Q17)</f>
+        <f>SUM(O6:O17)</f>
         <v/>
       </c>
     </row>
@@ -3871,11 +3659,11 @@
         <v/>
       </c>
       <c r="C22" s="55">
-        <f>SUM(K6:K17)</f>
+        <f>SUM(J6:J17)</f>
         <v/>
       </c>
       <c r="D22" s="55">
-        <f>SUM(R6:R17)</f>
+        <f>SUM(P6:P17)</f>
         <v/>
       </c>
     </row>
@@ -3890,11 +3678,11 @@
         <v/>
       </c>
       <c r="C23" s="55">
-        <f>SUM(L6:L17)</f>
+        <f>SUM(K6:K17)</f>
         <v/>
       </c>
       <c r="D23" s="55">
-        <f>SUM(S6:S17)</f>
+        <f>SUM(Q6:Q17)</f>
         <v/>
       </c>
     </row>
@@ -3909,11 +3697,11 @@
         <v/>
       </c>
       <c r="C24" s="53">
-        <f>SUM(M6:M17)</f>
+        <f>SUM(L6:L17)</f>
         <v/>
       </c>
       <c r="D24" s="53">
-        <f>SUM(T6:T17)</f>
+        <f>SUM(R6:R17)</f>
         <v/>
       </c>
     </row>
@@ -3924,15 +3712,15 @@
         </is>
       </c>
       <c r="B25" s="57">
-        <f>(SUMPRODUCT(C6:C17,Assumptions!$B$5)+SUMPRODUCT(D6:D17,Assumptions!$B$6))*Assumptions!$B$19+(SUMPRODUCT(E6:E17,Assumptions!$B$7))*Assumptions!$B$20-12*Assumptions!$B$21</f>
+        <f>(SUMPRODUCT(C6:C17,Assumptions!$B$5)+SUMPRODUCT(D6:D17,Assumptions!$B$6))*Assumptions!$B$20+(SUMPRODUCT(E6:E17,Assumptions!$B$7))*Assumptions!$B$21-12*Assumptions!$B$22</f>
         <v/>
       </c>
       <c r="C25" s="57">
-        <f>(SUMPRODUCT(J6:J17,Assumptions!$B$5)+SUMPRODUCT(K6:K17,Assumptions!$B$6))*Assumptions!$B$19+(SUMPRODUCT(L6:L17,Assumptions!$B$7))*Assumptions!$B$20-12*Assumptions!$B$21</f>
+        <f>(SUMPRODUCT(I6:I17,Assumptions!$B$5)+SUMPRODUCT(J6:J17,Assumptions!$B$6))*Assumptions!$B$20+(SUMPRODUCT(K6:K17,Assumptions!$B$7))*Assumptions!$B$21-12*Assumptions!$B$22</f>
         <v/>
       </c>
       <c r="D25" s="57">
-        <f>(SUMPRODUCT(Q6:Q17,Assumptions!$B$5)+SUMPRODUCT(R6:R17,Assumptions!$B$6))*Assumptions!$B$19+(SUMPRODUCT(S6:S17,Assumptions!$B$7))*Assumptions!$B$20-12*Assumptions!$B$21</f>
+        <f>(SUMPRODUCT(O6:O17,Assumptions!$B$5)+SUMPRODUCT(P6:P17,Assumptions!$B$6))*Assumptions!$B$20+(SUMPRODUCT(Q6:Q17,Assumptions!$B$7))*Assumptions!$B$21-12*Assumptions!$B$22</f>
         <v/>
       </c>
     </row>
@@ -3947,29 +3735,48 @@
         <v/>
       </c>
       <c r="C26" s="54">
-        <f>MAX(N6:N17)</f>
+        <f>MAX(M6:M17)</f>
         <v/>
       </c>
       <c r="D26" s="54">
-        <f>MAX(U6:U17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="40" customHeight="1" s="21">
-      <c r="A28" s="45" t="inlineStr">
-        <is>
-          <t>Margins and overhead are working estimates from the business plan (90% audit/self margin, 65% hardening margin, $223/mo fixed overhead) — not a full P&amp;L. Treat this as a directional comparison across scenarios, not a substitute for the month-by-month model in the business plan.</t>
+        <f>MAX(S6:S17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="51" t="inlineStr">
+        <is>
+          <t>Capacity Threshold (Peak Month, hrs/wk)</t>
+        </is>
+      </c>
+      <c r="B27" s="54">
+        <f>IF(12&gt;=Assumptions!$B$19,Assumptions!$B$18,Assumptions!$B$17)</f>
+        <v/>
+      </c>
+      <c r="C27" s="54">
+        <f>Assumptions!$B$17</f>
+        <v/>
+      </c>
+      <c r="D27" s="54">
+        <f>Assumptions!$B$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="55" customHeight="1" s="21">
+      <c r="A29" s="45" t="inlineStr">
+        <is>
+          <t>Path A's threshold uses Month 12 (post-join) for comparison since that's the relevant capacity once the partner is in full-time; check earlier months against the solo rate if you want the pre-join capacity picture. Legal note: Path C drops hardening entirely, which means almost every open item in legal-risk-notes.md (contractor-licensing exemption, permits, marketing-as-contractor risk) becomes moot — there's no physical contracting work to license at all.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="Q4:V4"/>
-    <mergeCell ref="C4:H4"/>
-    <mergeCell ref="A2:T2"/>
-    <mergeCell ref="J4:O4"/>
-    <mergeCell ref="A28:J28"/>
+    <mergeCell ref="I4:M4"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="A29:L29"/>
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="A2:S2"/>
+    <mergeCell ref="O4:S4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Drop A/B/C labeling, add itemized costs and marketing spend per scenario
</commit_message>
<xml_diff>
--- a/business/growth-poam.xlsx
+++ b/business/growth-poam.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth Curve" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POAM" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Business Model Paths" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -230,7 +230,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -394,6 +394,14 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="13" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -647,11 +655,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="48" customWidth="1" style="20" min="1" max="1"/>
     <col width="16" customWidth="1" style="20" min="2" max="2"/>
+    <col width="42" customWidth="1" style="21" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.35" customHeight="1" s="21">
@@ -775,7 +784,7 @@
     <row r="17">
       <c r="A17" s="30" t="inlineStr">
         <is>
-          <t>Solo Part-Time Hours / Week (evenings, Paths B &amp; C, and Path A before partner joins)</t>
+          <t>Solo Part-Time Hours / Week (evenings)</t>
         </is>
       </c>
       <c r="B17" s="63" t="n">
@@ -785,7 +794,7 @@
     <row r="18">
       <c r="A18" s="30" t="inlineStr">
         <is>
-          <t>Two-Person Full-Time Hours / Week (Path A, after partner joins)</t>
+          <t>Two-Person Full-Time Hours / Week (once a partner joins)</t>
         </is>
       </c>
       <c r="B18" s="63" t="n">
@@ -795,7 +804,7 @@
     <row r="19">
       <c r="A19" s="30" t="inlineStr">
         <is>
-          <t>Partner Join Month (Path A trigger, 1-12)</t>
+          <t>Partner Join Month (1-12, for the 'Partner Goes Full-Time' scenario)</t>
         </is>
       </c>
       <c r="B19" s="63" t="n">
@@ -823,25 +832,159 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="30" t="inlineStr">
-        <is>
-          <t>Fixed Monthly Overhead ($)</t>
-        </is>
-      </c>
-      <c r="B22" s="33" t="n">
-        <v>223</v>
+      <c r="A22" s="29" t="inlineStr">
+        <is>
+          <t>Fixed Monthly Overhead (itemized)</t>
+        </is>
+      </c>
+      <c r="B22" s="73" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="30" t="inlineStr">
+        <is>
+          <t>GL + E&amp;O Insurance ($/mo)</t>
+        </is>
+      </c>
+      <c r="B23" s="33" t="n">
+        <v>145</v>
       </c>
     </row>
     <row r="24" ht="55" customHeight="1" s="21">
-      <c r="A24" s="45" t="inlineStr">
-        <is>
-          <t>These three paths are the actual decision on the table, not just optimism levels. Path A assumes your business partner leaves their job once volume justifies it (Month 19 sets when); Path B keeps this a permanent evenings/weekends operation; Path C also stays part-time solo but drops the hardening add-on entirely, which sidesteps almost every open item in legal-risk-notes.md since there's no contractor-licensing exemption being relied on.</t>
+      <c r="A24" s="74" t="inlineStr">
+        <is>
+          <t>Tech Stack ($/mo)</t>
+        </is>
+      </c>
+      <c r="B24" s="33" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>Google Workspace ($/mo)</t>
+        </is>
+      </c>
+      <c r="B25" s="33" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="75" t="inlineStr">
+        <is>
+          <t>Total Fixed Overhead ($/mo)</t>
+        </is>
+      </c>
+      <c r="B26" s="76">
+        <f>SUM(B23:B25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="29" t="inlineStr">
+        <is>
+          <t>Marketing Channel Menu (reference — typical monthly cost, from the business plan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="75" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="B29" s="75" t="inlineStr">
+        <is>
+          <t>Typical $/mo</t>
+        </is>
+      </c>
+      <c r="C29" s="75" t="inlineStr">
+        <is>
+          <t>What it's meant to produce</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>Direct mail (Radius Blitz postcards)</t>
+        </is>
+      </c>
+      <c r="B30" s="33" t="n">
+        <v>200</v>
+      </c>
+      <c r="C30" s="77" t="inlineStr">
+        <is>
+          <t>300-500 postcards per active job</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>Lawn signage / worksite banners</t>
+        </is>
+      </c>
+      <c r="B31" s="33" t="n">
+        <v>25</v>
+      </c>
+      <c r="C31" s="77" t="inlineStr">
+        <is>
+          <t>~$100 one-time, spread over ~4 months</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Nextdoor Verified Sponsorship</t>
+        </is>
+      </c>
+      <c r="B32" s="33" t="n">
+        <v>65</v>
+      </c>
+      <c r="C32" s="77" t="inlineStr">
+        <is>
+          <t>Local sponsorship in target ZIP codes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>Events &amp; trade show booths</t>
+        </is>
+      </c>
+      <c r="B33" s="33" t="n">
+        <v>33</v>
+      </c>
+      <c r="C33" s="77" t="inlineStr">
+        <is>
+          <t>~$300-500/yr, 2-3 regional fairs</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="75" t="inlineStr">
+        <is>
+          <t>Sum of all channels above ($/mo)</t>
+        </is>
+      </c>
+      <c r="B34" s="76">
+        <f>SUM(B30:B33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="55" customHeight="1" s="21">
+      <c r="A36" s="45" t="inlineStr">
+        <is>
+          <t>This menu is a reference, not wired into the scenarios automatically — marketing effectiveness is too uncertain to model precisely. Each scenario on the Scenarios tab has its own editable Monthly Marketing Spend cell; use this menu to decide what mix of channels that number represents, then adjust the scenario's audit/self/hardening volumes to reflect what you think that spend buys.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A36:F36"/>
     <mergeCell ref="A14:F14"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -1456,7 +1599,7 @@
       </c>
       <c r="C4" s="64" t="inlineStr">
         <is>
-          <t>Decide operating path: (A) partner joins full-time once volume justifies it, (B) permanent part-time evenings solo, or (C) homeowner-inspections-only solo part-time (no hardening add-on)</t>
+          <t>Decide operating model: a business partner joining full-time once volume justifies it, a permanent part-time evenings-only operation, or a part-time homeowner-inspections-only business (no hardening add-on)</t>
         </is>
       </c>
       <c r="D4" s="64" t="inlineStr">
@@ -1486,7 +1629,7 @@
       </c>
       <c r="I4" s="64" t="inlineStr">
         <is>
-          <t>Decision documented — see 'Business Model Paths' tab. Determines whether hardening-related POAM items (1.3, 2.1) and legal-risk items 1/2/5/6 are even relevant.</t>
+          <t>Decision documented — see the Scenarios tab. Determines whether hardening-related POAM items (1.3, 2.1) and legal-risk items 1/2/5/6 are even relevant.</t>
         </is>
       </c>
     </row>
@@ -2737,7 +2880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S29"/>
+  <dimension ref="A1:S31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="21" min="1" max="1"/>
@@ -2765,31 +2908,31 @@
     <row r="1">
       <c r="A1" s="44" t="inlineStr">
         <is>
-          <t>Which Path — Partner Joins Full-Time / Part-Time Evenings / Homeowner-Only</t>
+          <t>Growth Scenarios — Compare Side by Side, Edit Any Number</t>
         </is>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1" s="21">
       <c r="A2" s="45" t="inlineStr">
         <is>
-          <t>Audits / Self / Hardening are editable per-path inputs (blue) — each path has a genuinely different volume story, not just a multiplier. Revenue, Hours/Week, and Capacity are formulas that recalc from the Assumptions tab.</t>
+          <t>Audits / Self / Hardening / Marketing Spend are editable inputs (blue) for each scenario. Everything else recalculates from the Assumptions tab. These three are starting points, not the only options — copy a block sideways on this sheet to add your own.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="C4" s="65" t="inlineStr">
         <is>
-          <t>A — PARTNER JOINS FULL-TIME</t>
+          <t>PARTNER GOES FULL-TIME</t>
         </is>
       </c>
       <c r="I4" s="65" t="inlineStr">
         <is>
-          <t>B — PART-TIME EVENINGS (SOLO, INDEFINITELY)</t>
+          <t>PART-TIME EVENINGS (SOLO)</t>
         </is>
       </c>
       <c r="O4" s="65" t="inlineStr">
         <is>
-          <t>C — HOMEOWNER INSPECTIONS ONLY (SOLO, PART-TIME, NO HARDENING)</t>
+          <t>HOMEOWNER INSPECTIONS ONLY (PART-TIME)</t>
         </is>
       </c>
     </row>
@@ -3606,6 +3749,9 @@
           <t>Year-1 Summary</t>
         </is>
       </c>
+      <c r="B19" s="30" t="n"/>
+      <c r="C19" s="30" t="n"/>
+      <c r="D19" s="30" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="47" t="inlineStr">
@@ -3615,17 +3761,17 @@
       </c>
       <c r="B20" s="47" t="inlineStr">
         <is>
-          <t>A — Partner Joins</t>
+          <t>Partner Goes Full-Time</t>
         </is>
       </c>
       <c r="C20" s="47" t="inlineStr">
         <is>
-          <t>B — Evenings Only</t>
+          <t>Part-Time Evenings</t>
         </is>
       </c>
       <c r="D20" s="47" t="inlineStr">
         <is>
-          <t>C — Homeowner-Only</t>
+          <t>Homeowner Inspections Only</t>
         </is>
       </c>
     </row>
@@ -3706,74 +3852,102 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="56" t="inlineStr">
+      <c r="A25" s="51" t="inlineStr">
+        <is>
+          <t>Monthly Marketing Spend ($)</t>
+        </is>
+      </c>
+      <c r="B25" s="78" t="n">
+        <v>200</v>
+      </c>
+      <c r="C25" s="78" t="n">
+        <v>50</v>
+      </c>
+      <c r="D25" s="78" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="56" t="inlineStr">
         <is>
           <t>Est. Year-1 Net Profit ($)</t>
         </is>
       </c>
-      <c r="B25" s="57">
-        <f>(SUMPRODUCT(C6:C17,Assumptions!$B$5)+SUMPRODUCT(D6:D17,Assumptions!$B$6))*Assumptions!$B$20+(SUMPRODUCT(E6:E17,Assumptions!$B$7))*Assumptions!$B$21-12*Assumptions!$B$22</f>
-        <v/>
-      </c>
-      <c r="C25" s="57">
-        <f>(SUMPRODUCT(I6:I17,Assumptions!$B$5)+SUMPRODUCT(J6:J17,Assumptions!$B$6))*Assumptions!$B$20+(SUMPRODUCT(K6:K17,Assumptions!$B$7))*Assumptions!$B$21-12*Assumptions!$B$22</f>
-        <v/>
-      </c>
-      <c r="D25" s="57">
-        <f>(SUMPRODUCT(O6:O17,Assumptions!$B$5)+SUMPRODUCT(P6:P17,Assumptions!$B$6))*Assumptions!$B$20+(SUMPRODUCT(Q6:Q17,Assumptions!$B$7))*Assumptions!$B$21-12*Assumptions!$B$22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="51" t="inlineStr">
-        <is>
-          <t>Peak Month Hours/Week</t>
-        </is>
-      </c>
-      <c r="B26" s="54">
-        <f>MAX(G6:G17)</f>
-        <v/>
-      </c>
-      <c r="C26" s="54">
-        <f>MAX(M6:M17)</f>
-        <v/>
-      </c>
-      <c r="D26" s="54">
-        <f>MAX(S6:S17)</f>
+      <c r="B26" s="57">
+        <f>(SUMPRODUCT(C6:C17,Assumptions!$B$5)+SUMPRODUCT(D6:D17,Assumptions!$B$6))*Assumptions!$B$20+(SUMPRODUCT(E6:E17,Assumptions!$B$7))*Assumptions!$B$21-12*Assumptions!$B$26-12*B25</f>
+        <v/>
+      </c>
+      <c r="C26" s="57">
+        <f>(SUMPRODUCT(I6:I17,Assumptions!$B$5)+SUMPRODUCT(J6:J17,Assumptions!$B$6))*Assumptions!$B$20+(SUMPRODUCT(K6:K17,Assumptions!$B$7))*Assumptions!$B$21-12*Assumptions!$B$26-12*C25</f>
+        <v/>
+      </c>
+      <c r="D26" s="57">
+        <f>(SUMPRODUCT(O6:O17,Assumptions!$B$5)+SUMPRODUCT(P6:P17,Assumptions!$B$6))*Assumptions!$B$20+(SUMPRODUCT(Q6:Q17,Assumptions!$B$7))*Assumptions!$B$21-12*Assumptions!$B$26-12*D25</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="51" t="inlineStr">
         <is>
+          <t>Peak Month Hours/Week</t>
+        </is>
+      </c>
+      <c r="B27" s="54">
+        <f>MAX(G6:G17)</f>
+        <v/>
+      </c>
+      <c r="C27" s="54">
+        <f>MAX(M6:M17)</f>
+        <v/>
+      </c>
+      <c r="D27" s="54">
+        <f>MAX(S6:S17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
           <t>Capacity Threshold (Peak Month, hrs/wk)</t>
         </is>
       </c>
-      <c r="B27" s="54">
+      <c r="B28" s="30">
         <f>IF(12&gt;=Assumptions!$B$19,Assumptions!$B$18,Assumptions!$B$17)</f>
         <v/>
       </c>
-      <c r="C27" s="54">
+      <c r="C28" s="30">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
-      <c r="D27" s="54">
+      <c r="D28" s="30">
         <f>Assumptions!$B$17</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="55" customHeight="1" s="21">
-      <c r="A29" s="45" t="inlineStr">
-        <is>
-          <t>Path A's threshold uses Month 12 (post-join) for comparison since that's the relevant capacity once the partner is in full-time; check earlier months against the solo rate if you want the pre-join capacity picture. Legal note: Path C drops hardening entirely, which means almost every open item in legal-risk-notes.md (contractor-licensing exemption, permits, marketing-as-contractor risk) becomes moot — there's no physical contracting work to license at all.</t>
-        </is>
-      </c>
+      <c r="A29" s="74" t="n"/>
+      <c r="B29" s="30" t="n"/>
+      <c r="C29" s="30" t="n"/>
+      <c r="D29" s="30" t="n"/>
+    </row>
+    <row r="30" ht="70" customHeight="1" s="21">
+      <c r="A30" s="45" t="inlineStr">
+        <is>
+          <t>The 'Partner Goes Full-Time' threshold uses Month 12 (post-join) for comparison, since that's the relevant capacity once the partner is in full-time — check earlier months against the solo rate for the pre-join picture. Legal note: 'Homeowner Inspections Only' drops hardening entirely, which means almost every open item in legal-risk-notes.md (contractor-licensing exemption, permits, marketing-as-contractor risk) becomes moot — there's no physical contracting work to license at all. Monthly Marketing Spend above is a flat monthly figure you set; see the Marketing Channel Menu on the Assumptions tab for what a given number typically buys.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="30" t="n"/>
+      <c r="B31" s="30" t="n"/>
+      <c r="C31" s="30" t="n"/>
+      <c r="D31" s="30" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="I4:M4"/>
+    <mergeCell ref="A30:L30"/>
     <mergeCell ref="C4:G4"/>
-    <mergeCell ref="A29:L29"/>
     <mergeCell ref="A1:S1"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="O4:S4"/>

</xml_diff>